<commit_message>
Limit conversion download to a single user details sheet
</commit_message>
<xml_diff>
--- a/public/templates/dashboard-download-headers.xlsx
+++ b/public/templates/dashboard-download-headers.xlsx
@@ -2,17 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rc43df3b0b12f4b5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转化用户明细" sheetId="2" r:id="R88700f95f7b84c54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前线索用户明细" sheetId="3" r:id="Rba95386b4afa4bd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外呼用户明细" sheetId="4" r:id="Rc7fc4e7d327946f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跟进用户明细" sheetId="5" r:id="R25ad08ed031d444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话记录明细" sheetId="6" r:id="Rc67a96ee9f024d94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预约记录明细" sheetId="7" r:id="R11c6d3389c244b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="体验课记录明细" sheetId="8" r:id="Ra7f80e72a28549ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支付订单明细" sheetId="9" r:id="Rb00927e625464067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原因用户明细" sheetId="10" r:id="R36ba208eb71540a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="筛选条件" sheetId="11" r:id="R45e0c247f13e4b0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rce525ced0b0a4a88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转化用户明细" sheetId="2" r:id="Ra5292841a38e4993"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前线索用户明细" sheetId="3" r:id="Rfde6c7fd43104831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外呼用户明细" sheetId="4" r:id="Rbe42d43eefea448a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跟进用户明细" sheetId="5" r:id="Ra286821e75f44d01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话记录明细" sheetId="6" r:id="Rce2d80f795774f1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预约记录明细" sheetId="7" r:id="R10f16e6e35cc407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支付订单明细" sheetId="8" r:id="R1b9c22a7b9134bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原因用户明细" sheetId="9" r:id="R6cfdff33777442a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="筛选条件" sheetId="10" r:id="R08965038ae134257"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -328,7 +327,7 @@
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="3" t="str">
-        <x:v>本文件为空白明细模板合集。每个入口下载下列明细表，并附“筛选条件”；全部明细均有用户 ID。</x:v>
+        <x:v>本文件为空白明细模板合集。转化总览仅下载“转化用户明细”一张表；其余入口按下表下载并附“筛选条件”。</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -352,7 +351,7 @@
         <x:v>conversion-details.xlsx</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
-        <x:v>转化用户明细、通话记录明细、预约记录明细、体验课记录明细、支付订单明细</x:v>
+        <x:v>仅转化用户明细（一张工作表，每用户一行）</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
@@ -448,7 +447,7 @@
     </x:row>
     <x:row r="21" ht="35" customHeight="1">
       <x:c r="A21" s="9" t="str">
-        <x:v>核对金额：只在支付订单明细中按币种求和。AOV＝金额÷订单数，人均实付＝金额÷支付用户数；L2S＝已支付用户数÷线索数。</x:v>
+        <x:v>核对金额：转化按用户实付金额合计求和，其他入口按订单金额求和，均按币种区分。AOV＝金额÷订单数；L2S＝已支付用户数÷线索数。</x:v>
       </x:c>
       <x:c r="B21" s="9"/>
       <x:c r="C21" s="9"/>
@@ -483,7 +482,7 @@
     </x:row>
     <x:row r="31" ht="35" customHeight="1">
       <x:c r="A31" s="9" t="str">
-        <x:v>关联：通过用户 ID 与记录 ID 核对，不把多个事件表多对多联表后累加金额。模板的首次/最近时间不代替全部记录明细。</x:v>
+        <x:v>转化下载：只包含转化用户明细；六项 0/1 标记核对人数，首次时间取有效记录。其他入口的多条业务记录按用户 ID 去重核对。</x:v>
       </x:c>
       <x:c r="B31" s="9"/>
       <x:c r="C31" s="9"/>
@@ -505,125 +504,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="48" customHeight="1">
-      <x:c r="A1" s="14" t="str">
-        <x:v>用户 ID</x:v>
-      </x:c>
-      <x:c r="B1" s="14" t="str">
-        <x:v>姓名</x:v>
-      </x:c>
-      <x:c r="C1" s="14" t="str">
-        <x:v>业务线</x:v>
-      </x:c>
-      <x:c r="D1" s="14" t="str">
-        <x:v>用户类型</x:v>
-      </x:c>
-      <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
-      </x:c>
-      <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
-      </x:c>
-      <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
-      </x:c>
-      <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
-      </x:c>
-      <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
-      </x:c>
-      <x:c r="J1" s="14" t="str">
-        <x:v>当前销售阶段</x:v>
-      </x:c>
-      <x:c r="K1" s="14" t="str">
-        <x:v>原因分类</x:v>
-      </x:c>
-      <x:c r="L1" s="14" t="str">
-        <x:v>具体原因</x:v>
-      </x:c>
-      <x:c r="M1" s="14" t="str">
-        <x:v>拒绝或结束时间</x:v>
-      </x:c>
-      <x:c r="N1" s="14" t="str">
-        <x:v>拒绝或结束日期</x:v>
-      </x:c>
-      <x:c r="O1" s="14" t="str">
-        <x:v>时间依据</x:v>
-      </x:c>
-      <x:c r="P1" s="14" t="str">
-        <x:v>最近跟进时间</x:v>
-      </x:c>
-      <x:c r="Q1" s="14" t="str">
-        <x:v>最近跟进备注</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="26" customHeight="1">
-      <x:c r="A2" s="15"/>
-      <x:c r="B2" s="4"/>
-      <x:c r="C2" s="4"/>
-      <x:c r="D2" s="4"/>
-      <x:c r="E2" s="4"/>
-      <x:c r="F2" s="4"/>
-      <x:c r="G2" s="4"/>
-      <x:c r="H2" s="4"/>
-      <x:c r="I2" s="4"/>
-      <x:c r="J2" s="4"/>
-      <x:c r="K2" s="4"/>
-      <x:c r="L2" s="4"/>
-      <x:c r="M2" s="4"/>
-      <x:c r="N2" s="4"/>
-      <x:c r="O2" s="4"/>
-      <x:c r="P2" s="4"/>
-      <x:c r="Q2" s="4"/>
-    </x:row>
-    <x:row r="3" ht="26" customHeight="1">
-      <x:c r="A3" s="15"/>
-      <x:c r="B3" s="4"/>
-      <x:c r="C3" s="4"/>
-      <x:c r="D3" s="4"/>
-      <x:c r="E3" s="4"/>
-      <x:c r="F3" s="4"/>
-      <x:c r="G3" s="4"/>
-      <x:c r="H3" s="4"/>
-      <x:c r="I3" s="4"/>
-      <x:c r="J3" s="4"/>
-      <x:c r="K3" s="4"/>
-      <x:c r="L3" s="4"/>
-      <x:c r="M3" s="4"/>
-      <x:c r="N3" s="4"/>
-      <x:c r="O3" s="4"/>
-      <x:c r="P3" s="4"/>
-      <x:c r="Q3" s="4"/>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1698,6 +1578,7 @@
     <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1729,31 +1610,34 @@
         <x:v>用户状态</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>课程记录 ID</x:v>
+        <x:v>订单 ID</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>课标</x:v>
+        <x:v>商品名称</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>课程名称</x:v>
+        <x:v>订单状态</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>课程类型</x:v>
+        <x:v>原价</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>课程状态</x:v>
+        <x:v>实付金额</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>老师</x:v>
+        <x:v>币种</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>上课时间</x:v>
+        <x:v>支付方式</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>完课时间</x:v>
+        <x:v>支付时间</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>完课日期</x:v>
+        <x:v>支付日期</x:v>
+      </x:c>
+      <x:c r="S1" s="14" t="str">
+        <x:v>有效期截止时间</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
@@ -1775,6 +1659,7 @@
       <x:c r="P2" s="4"/>
       <x:c r="Q2" s="4"/>
       <x:c r="R2" s="4"/>
+      <x:c r="S2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -1795,6 +1680,7 @@
       <x:c r="P3" s="4"/>
       <x:c r="Q3" s="4"/>
       <x:c r="R3" s="4"/>
+      <x:c r="S3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1822,8 +1708,6 @@
     <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1855,34 +1739,28 @@
         <x:v>用户状态</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>订单 ID</x:v>
+        <x:v>当前销售阶段</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>商品名称</x:v>
+        <x:v>原因分类</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>订单状态</x:v>
+        <x:v>具体原因</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>原价</x:v>
+        <x:v>拒绝或结束时间</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>实付金额</x:v>
+        <x:v>拒绝或结束日期</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>币种</x:v>
+        <x:v>时间依据</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>支付方式</x:v>
+        <x:v>最近跟进时间</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>支付时间</x:v>
-      </x:c>
-      <x:c r="R1" s="14" t="str">
-        <x:v>支付日期</x:v>
-      </x:c>
-      <x:c r="S1" s="14" t="str">
-        <x:v>有效期截止时间</x:v>
+        <x:v>最近跟进备注</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
@@ -1895,7 +1773,7 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="4"/>
-      <x:c r="J2" s="15"/>
+      <x:c r="J2" s="4"/>
       <x:c r="K2" s="4"/>
       <x:c r="L2" s="4"/>
       <x:c r="M2" s="4"/>
@@ -1903,8 +1781,6 @@
       <x:c r="O2" s="4"/>
       <x:c r="P2" s="4"/>
       <x:c r="Q2" s="4"/>
-      <x:c r="R2" s="4"/>
-      <x:c r="S2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -1916,7 +1792,7 @@
       <x:c r="G3" s="4"/>
       <x:c r="H3" s="4"/>
       <x:c r="I3" s="4"/>
-      <x:c r="J3" s="15"/>
+      <x:c r="J3" s="4"/>
       <x:c r="K3" s="4"/>
       <x:c r="L3" s="4"/>
       <x:c r="M3" s="4"/>
@@ -1924,8 +1800,6 @@
       <x:c r="O3" s="4"/>
       <x:c r="P3" s="4"/>
       <x:c r="Q3" s="4"/>
-      <x:c r="R3" s="4"/>
-      <x:c r="S3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Keep only primary detail sheet in all dashboard downloads
</commit_message>
<xml_diff>
--- a/public/templates/dashboard-download-headers.xlsx
+++ b/public/templates/dashboard-download-headers.xlsx
@@ -2,16 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rce525ced0b0a4a88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转化用户明细" sheetId="2" r:id="Ra5292841a38e4993"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前线索用户明细" sheetId="3" r:id="Rfde6c7fd43104831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外呼用户明细" sheetId="4" r:id="Rbe42d43eefea448a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跟进用户明细" sheetId="5" r:id="Ra286821e75f44d01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话记录明细" sheetId="6" r:id="Rce2d80f795774f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预约记录明细" sheetId="7" r:id="R10f16e6e35cc407c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支付订单明细" sheetId="8" r:id="R1b9c22a7b9134bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原因用户明细" sheetId="9" r:id="R6cfdff33777442a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="筛选条件" sheetId="10" r:id="R08965038ae134257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rd9c3b3f5de874c1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转化用户明细" sheetId="2" r:id="R8902cf60a1314410"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前线索用户明细" sheetId="3" r:id="R87747ec1507e4e00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外呼用户明细" sheetId="4" r:id="R908c551b5e364f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跟进用户明细" sheetId="5" r:id="R0ef41c56d8b64514"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话记录明细" sheetId="6" r:id="R0d4e04d13357455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支付订单明细" sheetId="7" r:id="R566da6b17cf84037"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原因用户明细" sheetId="8" r:id="R1543de9247e9469e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -77,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -112,7 +110,6 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -327,7 +324,7 @@
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="3" t="str">
-        <x:v>本文件为空白明细模板合集。转化总览仅下载“转化用户明细”一张表；其余入口按下表下载并附“筛选条件”。</x:v>
+        <x:v>本文件是各入口的空白表头合集。实际每次下载一个 Excel，且只包含下表对应的一张明细表。</x:v>
       </x:c>
       <x:c r="B4" s="3"/>
       <x:c r="C4" s="3"/>
@@ -373,7 +370,7 @@
         <x:v>followup-calls.xlsx</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
-        <x:v>外呼用户明细、通话记录明细</x:v>
+        <x:v>外呼用户明细</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
@@ -384,7 +381,7 @@
         <x:v>followup-followup.xlsx</x:v>
       </x:c>
       <x:c r="C10" s="6" t="str">
-        <x:v>跟进用户明细、预约记录明细、支付订单明细</x:v>
+        <x:v>跟进用户明细</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
@@ -433,7 +430,7 @@
     </x:row>
     <x:row r="17" ht="35" customHeight="1">
       <x:c r="A17" s="9" t="str">
-        <x:v>每行含义：用户明细每用户一行；通话、预约、课程、支付明细每条业务记录一行，同一用户可有多行。</x:v>
+        <x:v>每行含义：用户明细每用户一行；通话、支付明细每条业务记录一行，同一用户可有多行。</x:v>
       </x:c>
       <x:c r="B17" s="9"/>
       <x:c r="C17" s="9"/>
@@ -447,14 +444,14 @@
     </x:row>
     <x:row r="21" ht="35" customHeight="1">
       <x:c r="A21" s="9" t="str">
-        <x:v>核对金额：转化按用户实付金额合计求和，其他入口按订单金额求和，均按币种区分。AOV＝金额÷订单数；L2S＝已支付用户数÷线索数。</x:v>
+        <x:v>核对金额：转化和跟进按用户实付金额合计求和，支付结果按订单金额求和，均按币种区分。AOV＝金额÷订单数；L2S＝已支付用户数÷线索数。</x:v>
       </x:c>
       <x:c r="B21" s="9"/>
       <x:c r="C21" s="9"/>
     </x:row>
     <x:row r="23" ht="35" customHeight="1">
       <x:c r="A23" s="9" t="str">
-        <x:v>时间：全部采用当前登录用户的浏览器时区，时间含时分秒及偏移量；筛选条件记录实际 IANA 时区。不固定 UTC+7。</x:v>
+        <x:v>时间：全部采用当前登录用户的浏览器时区，时间含时分秒及偏移量。不固定 UTC+7。</x:v>
       </x:c>
       <x:c r="B23" s="9"/>
       <x:c r="C23" s="9"/>
@@ -482,7 +479,7 @@
     </x:row>
     <x:row r="31" ht="35" customHeight="1">
       <x:c r="A31" s="9" t="str">
-        <x:v>转化下载：只包含转化用户明细；六项 0/1 标记核对人数，首次时间取有效记录。其他入口的多条业务记录按用户 ID 去重核对。</x:v>
+        <x:v>所有下载：只保留原来的第一张明细表，名称、字段和明细值保持不变；不附加其他业务记录表或筛选条件表。</x:v>
       </x:c>
       <x:c r="B31" s="9"/>
       <x:c r="C31" s="9"/>
@@ -499,111 +496,6 @@
     <x:mergeCell ref="A29:C29"/>
     <x:mergeCell ref="A31:C31"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="80" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="11" t="str">
-        <x:v>项目</x:v>
-      </x:c>
-      <x:c r="B1" s="11" t="str">
-        <x:v>内容</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="4" t="str">
-        <x:v>下载模块</x:v>
-      </x:c>
-      <x:c r="B2" s="4"/>
-    </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="4" t="str">
-        <x:v>所选业务线</x:v>
-      </x:c>
-      <x:c r="B3" s="4"/>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="4" t="str">
-        <x:v>授权范围内的业务线</x:v>
-      </x:c>
-      <x:c r="B4" s="4"/>
-    </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="4" t="str">
-        <x:v>已选 CC</x:v>
-      </x:c>
-      <x:c r="B5" s="4"/>
-    </x:row>
-    <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="4" t="str">
-        <x:v>CC 账号</x:v>
-      </x:c>
-      <x:c r="B6" s="4"/>
-    </x:row>
-    <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="4" t="str">
-        <x:v>日期范围／日期口径（按入口）</x:v>
-      </x:c>
-      <x:c r="B7" s="4"/>
-    </x:row>
-    <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="4" t="str">
-        <x:v>一级分组／分组方式</x:v>
-      </x:c>
-      <x:c r="B8" s="4"/>
-    </x:row>
-    <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="4" t="str">
-        <x:v>二级分组（适用时）</x:v>
-      </x:c>
-      <x:c r="B9" s="4"/>
-    </x:row>
-    <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="4" t="str">
-        <x:v>用户范围</x:v>
-      </x:c>
-      <x:c r="B10" s="4"/>
-    </x:row>
-    <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="4" t="str">
-        <x:v>统计时区</x:v>
-      </x:c>
-      <x:c r="B11" s="4"/>
-    </x:row>
-    <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="4" t="str">
-        <x:v>页面统计时间</x:v>
-      </x:c>
-      <x:c r="B12" s="4"/>
-    </x:row>
-    <x:row r="13" ht="28" customHeight="1">
-      <x:c r="A13" s="4" t="str">
-        <x:v>导出时间</x:v>
-      </x:c>
-      <x:c r="B13" s="4"/>
-    </x:row>
-    <x:row r="14" ht="28" customHeight="1">
-      <x:c r="A14" s="4" t="str">
-        <x:v>下载范围</x:v>
-      </x:c>
-      <x:c r="B14" s="4"/>
-    </x:row>
-    <x:row r="15" ht="28" customHeight="1">
-      <x:c r="A15" s="4" t="str">
-        <x:v>合计核对</x:v>
-      </x:c>
-      <x:c r="B15" s="4"/>
-    </x:row>
-  </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -1436,8 +1328,6 @@
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1469,40 +1359,34 @@
         <x:v>用户状态</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>预约 ID</x:v>
+        <x:v>订单 ID</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>预约创建时间</x:v>
+        <x:v>商品名称</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>预约上课时间</x:v>
+        <x:v>订单状态</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>预约上课日期</x:v>
+        <x:v>原价</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>预约状态</x:v>
+        <x:v>实付金额</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>出勤状态</x:v>
+        <x:v>币种</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>咨询状态</x:v>
+        <x:v>支付方式</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>原因</x:v>
+        <x:v>支付时间</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>预约备注</x:v>
+        <x:v>支付日期</x:v>
       </x:c>
       <x:c r="S1" s="14" t="str">
-        <x:v>创建人</x:v>
-      </x:c>
-      <x:c r="T1" s="14" t="str">
-        <x:v>更新时间</x:v>
-      </x:c>
-      <x:c r="U1" s="14" t="str">
-        <x:v>更新人</x:v>
+        <x:v>有效期截止时间</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
@@ -1525,8 +1409,6 @@
       <x:c r="Q2" s="4"/>
       <x:c r="R2" s="4"/>
       <x:c r="S2" s="4"/>
-      <x:c r="T2" s="4"/>
-      <x:c r="U2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -1548,8 +1430,6 @@
       <x:c r="Q3" s="4"/>
       <x:c r="R3" s="4"/>
       <x:c r="S3" s="4"/>
-      <x:c r="T3" s="4"/>
-      <x:c r="U3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1577,137 +1457,6 @@
     <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="48" customHeight="1">
-      <x:c r="A1" s="14" t="str">
-        <x:v>用户 ID</x:v>
-      </x:c>
-      <x:c r="B1" s="14" t="str">
-        <x:v>姓名</x:v>
-      </x:c>
-      <x:c r="C1" s="14" t="str">
-        <x:v>业务线</x:v>
-      </x:c>
-      <x:c r="D1" s="14" t="str">
-        <x:v>用户类型</x:v>
-      </x:c>
-      <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
-      </x:c>
-      <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
-      </x:c>
-      <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
-      </x:c>
-      <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
-      </x:c>
-      <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
-      </x:c>
-      <x:c r="J1" s="14" t="str">
-        <x:v>订单 ID</x:v>
-      </x:c>
-      <x:c r="K1" s="14" t="str">
-        <x:v>商品名称</x:v>
-      </x:c>
-      <x:c r="L1" s="14" t="str">
-        <x:v>订单状态</x:v>
-      </x:c>
-      <x:c r="M1" s="14" t="str">
-        <x:v>原价</x:v>
-      </x:c>
-      <x:c r="N1" s="14" t="str">
-        <x:v>实付金额</x:v>
-      </x:c>
-      <x:c r="O1" s="14" t="str">
-        <x:v>币种</x:v>
-      </x:c>
-      <x:c r="P1" s="14" t="str">
-        <x:v>支付方式</x:v>
-      </x:c>
-      <x:c r="Q1" s="14" t="str">
-        <x:v>支付时间</x:v>
-      </x:c>
-      <x:c r="R1" s="14" t="str">
-        <x:v>支付日期</x:v>
-      </x:c>
-      <x:c r="S1" s="14" t="str">
-        <x:v>有效期截止时间</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="26" customHeight="1">
-      <x:c r="A2" s="15"/>
-      <x:c r="B2" s="4"/>
-      <x:c r="C2" s="4"/>
-      <x:c r="D2" s="4"/>
-      <x:c r="E2" s="4"/>
-      <x:c r="F2" s="4"/>
-      <x:c r="G2" s="4"/>
-      <x:c r="H2" s="4"/>
-      <x:c r="I2" s="4"/>
-      <x:c r="J2" s="15"/>
-      <x:c r="K2" s="4"/>
-      <x:c r="L2" s="4"/>
-      <x:c r="M2" s="4"/>
-      <x:c r="N2" s="4"/>
-      <x:c r="O2" s="4"/>
-      <x:c r="P2" s="4"/>
-      <x:c r="Q2" s="4"/>
-      <x:c r="R2" s="4"/>
-      <x:c r="S2" s="4"/>
-    </x:row>
-    <x:row r="3" ht="26" customHeight="1">
-      <x:c r="A3" s="15"/>
-      <x:c r="B3" s="4"/>
-      <x:c r="C3" s="4"/>
-      <x:c r="D3" s="4"/>
-      <x:c r="E3" s="4"/>
-      <x:c r="F3" s="4"/>
-      <x:c r="G3" s="4"/>
-      <x:c r="H3" s="4"/>
-      <x:c r="I3" s="4"/>
-      <x:c r="J3" s="15"/>
-      <x:c r="K3" s="4"/>
-      <x:c r="L3" s="4"/>
-      <x:c r="M3" s="4"/>
-      <x:c r="N3" s="4"/>
-      <x:c r="O3" s="4"/>
-      <x:c r="P3" s="4"/>
-      <x:c r="Q3" s="4"/>
-      <x:c r="R3" s="4"/>
-      <x:c r="S3" s="4"/>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">

</xml_diff>

<commit_message>
Remove redundant current CC column from dashboard details
</commit_message>
<xml_diff>
--- a/public/templates/dashboard-download-headers.xlsx
+++ b/public/templates/dashboard-download-headers.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rd9c3b3f5de874c1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转化用户明细" sheetId="2" r:id="R8902cf60a1314410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前线索用户明细" sheetId="3" r:id="R87747ec1507e4e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外呼用户明细" sheetId="4" r:id="R908c551b5e364f75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跟进用户明细" sheetId="5" r:id="R0ef41c56d8b64514"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话记录明细" sheetId="6" r:id="R0d4e04d13357455d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支付订单明细" sheetId="7" r:id="R566da6b17cf84037"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原因用户明细" sheetId="8" r:id="R1543de9247e9469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R892fd86396da4be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转化用户明细" sheetId="2" r:id="R47b335a6b6814942"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前线索用户明细" sheetId="3" r:id="R3c7fc65dd07846a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外呼用户明细" sheetId="4" r:id="R56c8317eec764419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跟进用户明细" sheetId="5" r:id="Rdd278c065ce94f28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话记录明细" sheetId="6" r:id="Rad831d28948049d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="支付订单明细" sheetId="7" r:id="Rb394026992db4da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原因用户明细" sheetId="8" r:id="R0a9090ae0be444d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -526,7 +526,6 @@
     <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="24" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -543,60 +542,57 @@
         <x:v>用户类型</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
+        <x:v>当前 CC 账号</x:v>
       </x:c>
       <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
+        <x:v>注册时间</x:v>
       </x:c>
       <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
+        <x:v>注册日期</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
+        <x:v>用户状态</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
+        <x:v>线索数（含已付费）（0/1）</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>线索数（含已付费）（0/1）</x:v>
+        <x:v>外呼人数（0/1）</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>外呼人数（0/1）</x:v>
+        <x:v>接通人数（0/1）</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>接通人数（0/1）</x:v>
+        <x:v>预约人数（0/1）</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>预约人数（0/1）</x:v>
+        <x:v>体验课完成人数（0/1）</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>体验课完成人数（0/1）</x:v>
+        <x:v>已支付人数（0/1）</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>已支付人数（0/1）</x:v>
+        <x:v>首次有效外呼时间</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>首次有效外呼时间</x:v>
+        <x:v>首次接通时间</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>首次接通时间</x:v>
+        <x:v>首次预约创建时间</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>首次预约创建时间</x:v>
+        <x:v>首次体验课完成时间</x:v>
       </x:c>
       <x:c r="S1" s="14" t="str">
-        <x:v>首次体验课完成时间</x:v>
+        <x:v>首次有效支付时间</x:v>
       </x:c>
       <x:c r="T1" s="14" t="str">
-        <x:v>首次有效支付时间</x:v>
+        <x:v>有效已支付订单数</x:v>
       </x:c>
       <x:c r="U1" s="14" t="str">
-        <x:v>有效已支付订单数</x:v>
+        <x:v>币种</x:v>
       </x:c>
       <x:c r="V1" s="14" t="str">
-        <x:v>币种</x:v>
-      </x:c>
-      <x:c r="W1" s="14" t="str">
         <x:v>用户实付金额合计</x:v>
       </x:c>
     </x:row>
@@ -623,7 +619,6 @@
       <x:c r="T2" s="4"/>
       <x:c r="U2" s="4"/>
       <x:c r="V2" s="4"/>
-      <x:c r="W2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -648,7 +643,6 @@
       <x:c r="T3" s="4"/>
       <x:c r="U3" s="4"/>
       <x:c r="V3" s="4"/>
-      <x:c r="W3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -677,7 +671,6 @@
     <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -694,48 +687,45 @@
         <x:v>用户类型</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
+        <x:v>当前 CC 账号</x:v>
       </x:c>
       <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
+        <x:v>注册时间</x:v>
       </x:c>
       <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
+        <x:v>注册日期</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
+        <x:v>用户状态</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
+        <x:v>当前销售阶段</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>当前销售阶段</x:v>
+        <x:v>跟进进度</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>跟进进度</x:v>
+        <x:v>最近跟进时间</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>最近跟进时间</x:v>
+        <x:v>最近跟进备注</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>最近跟进备注</x:v>
+        <x:v>当前销售线索（0/1）</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>当前销售线索（0/1）</x:v>
+        <x:v>已分配（0/1）</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>已分配（0/1）</x:v>
+        <x:v>未分配（0/1）</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>未分配（0/1）</x:v>
+        <x:v>已拒绝（0/1）</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>已拒绝（0/1）</x:v>
+        <x:v>已结束（0/1）</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>已结束（0/1）</x:v>
-      </x:c>
-      <x:c r="S1" s="14" t="str">
         <x:v>暂不跟进（0/1）</x:v>
       </x:c>
     </x:row>
@@ -758,7 +748,6 @@
       <x:c r="P2" s="4"/>
       <x:c r="Q2" s="4"/>
       <x:c r="R2" s="4"/>
-      <x:c r="S2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -779,7 +768,6 @@
       <x:c r="P3" s="4"/>
       <x:c r="Q3" s="4"/>
       <x:c r="R3" s="4"/>
-      <x:c r="S3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -811,7 +799,6 @@
     <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -828,57 +815,54 @@
         <x:v>用户类型</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
+        <x:v>当前 CC 账号</x:v>
       </x:c>
       <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
+        <x:v>注册时间</x:v>
       </x:c>
       <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
+        <x:v>注册日期</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
+        <x:v>用户状态</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
+        <x:v>当前销售阶段</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>当前销售阶段</x:v>
+        <x:v>跟进进度</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>跟进进度</x:v>
+        <x:v>最近跟进时间</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>最近跟进时间</x:v>
+        <x:v>最近跟进备注</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>最近跟进备注</x:v>
+        <x:v>待外呼（0/1）</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>待外呼（0/1）</x:v>
+        <x:v>未接通 · 待跟进（0/1）</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>未接通 · 待跟进（0/1）</x:v>
+        <x:v>已拒绝（0/1）</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>已拒绝（0/1）</x:v>
+        <x:v>外呼人数（0/1）</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>外呼人数（0/1）</x:v>
+        <x:v>接通人数（0/1）</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>接通人数（0/1）</x:v>
+        <x:v>期间首次外呼时间</x:v>
       </x:c>
       <x:c r="S1" s="14" t="str">
-        <x:v>期间首次外呼时间</x:v>
+        <x:v>期间最近外呼时间</x:v>
       </x:c>
       <x:c r="T1" s="14" t="str">
-        <x:v>期间最近外呼时间</x:v>
+        <x:v>期间首次接通时间</x:v>
       </x:c>
       <x:c r="U1" s="14" t="str">
-        <x:v>期间首次接通时间</x:v>
-      </x:c>
-      <x:c r="V1" s="14" t="str">
         <x:v>期间最近接通时间</x:v>
       </x:c>
     </x:row>
@@ -904,7 +888,6 @@
       <x:c r="S2" s="4"/>
       <x:c r="T2" s="4"/>
       <x:c r="U2" s="4"/>
-      <x:c r="V2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -928,7 +911,6 @@
       <x:c r="S3" s="4"/>
       <x:c r="T3" s="4"/>
       <x:c r="U3" s="4"/>
-      <x:c r="V3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -968,7 +950,6 @@
     <x:col min="27" max="27" width="24" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="24" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="24" hidden="0" customWidth="1"/>
-    <x:col min="30" max="30" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -985,81 +966,78 @@
         <x:v>用户类型</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
+        <x:v>当前 CC 账号</x:v>
       </x:c>
       <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
+        <x:v>注册时间</x:v>
       </x:c>
       <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
+        <x:v>注册日期</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
+        <x:v>用户状态</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
+        <x:v>当前销售阶段</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>当前销售阶段</x:v>
+        <x:v>跟进进度</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>跟进进度</x:v>
+        <x:v>最近跟进时间</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>最近跟进时间</x:v>
+        <x:v>最近跟进备注</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>最近跟进备注</x:v>
+        <x:v>待预约（0/1）</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>待预约（0/1）</x:v>
+        <x:v>已预约（0/1）</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>已预约（0/1）</x:v>
+        <x:v>未出勤（0/1）</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>未出勤（0/1）</x:v>
+        <x:v>咨询未完成（0/1）</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>咨询未完成（0/1）</x:v>
+        <x:v>咨询已完成（0/1）</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>咨询已完成（0/1）</x:v>
+        <x:v>已结束（0/1）</x:v>
       </x:c>
       <x:c r="S1" s="14" t="str">
-        <x:v>已结束（0/1）</x:v>
+        <x:v>已支付（0/1）</x:v>
       </x:c>
       <x:c r="T1" s="14" t="str">
-        <x:v>已支付（0/1）</x:v>
+        <x:v>状态统计口径</x:v>
       </x:c>
       <x:c r="U1" s="14" t="str">
-        <x:v>状态统计口径</x:v>
+        <x:v>状态业务日期</x:v>
       </x:c>
       <x:c r="V1" s="14" t="str">
-        <x:v>状态业务日期</x:v>
+        <x:v>状态业务时间</x:v>
       </x:c>
       <x:c r="W1" s="14" t="str">
-        <x:v>状态业务时间</x:v>
+        <x:v>状态时间依据</x:v>
       </x:c>
       <x:c r="X1" s="14" t="str">
-        <x:v>状态时间依据</x:v>
+        <x:v>关联预约 ID</x:v>
       </x:c>
       <x:c r="Y1" s="14" t="str">
-        <x:v>关联预约 ID</x:v>
+        <x:v>期间首次支付时间</x:v>
       </x:c>
       <x:c r="Z1" s="14" t="str">
-        <x:v>期间首次支付时间</x:v>
+        <x:v>期间最近支付时间</x:v>
       </x:c>
       <x:c r="AA1" s="14" t="str">
-        <x:v>期间最近支付时间</x:v>
+        <x:v>有效已支付订单数</x:v>
       </x:c>
       <x:c r="AB1" s="14" t="str">
-        <x:v>有效已支付订单数</x:v>
+        <x:v>币种</x:v>
       </x:c>
       <x:c r="AC1" s="14" t="str">
-        <x:v>币种</x:v>
-      </x:c>
-      <x:c r="AD1" s="14" t="str">
         <x:v>用户实付金额合计</x:v>
       </x:c>
     </x:row>
@@ -1087,13 +1065,12 @@
       <x:c r="U2" s="4"/>
       <x:c r="V2" s="4"/>
       <x:c r="W2" s="4"/>
-      <x:c r="X2" s="4"/>
-      <x:c r="Y2" s="15"/>
+      <x:c r="X2" s="15"/>
+      <x:c r="Y2" s="4"/>
       <x:c r="Z2" s="4"/>
       <x:c r="AA2" s="4"/>
       <x:c r="AB2" s="4"/>
       <x:c r="AC2" s="4"/>
-      <x:c r="AD2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -1119,13 +1096,12 @@
       <x:c r="U3" s="4"/>
       <x:c r="V3" s="4"/>
       <x:c r="W3" s="4"/>
-      <x:c r="X3" s="4"/>
-      <x:c r="Y3" s="15"/>
+      <x:c r="X3" s="15"/>
+      <x:c r="Y3" s="4"/>
       <x:c r="Z3" s="4"/>
       <x:c r="AA3" s="4"/>
       <x:c r="AB3" s="4"/>
       <x:c r="AC3" s="4"/>
-      <x:c r="AD3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1161,7 +1137,6 @@
     <x:col min="23" max="23" width="24" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="24" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="24" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1178,69 +1153,66 @@
         <x:v>用户类型</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
+        <x:v>当前 CC 账号</x:v>
       </x:c>
       <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
+        <x:v>注册时间</x:v>
       </x:c>
       <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
+        <x:v>注册日期</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
+        <x:v>用户状态</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
+        <x:v>通话 ID</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>通话 ID</x:v>
+        <x:v>外呼系统</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>外呼系统</x:v>
+        <x:v>第三方通话 ID</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>第三方通话 ID</x:v>
+        <x:v>线路 ID</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>线路 ID</x:v>
+        <x:v>线路名称</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>线路名称</x:v>
+        <x:v>坐席</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>坐席</x:v>
+        <x:v>操作人</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>操作人</x:v>
+        <x:v>起呼时间</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>起呼时间</x:v>
+        <x:v>通话日期</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>通话日期</x:v>
+        <x:v>接通时间</x:v>
       </x:c>
       <x:c r="S1" s="14" t="str">
-        <x:v>接通时间</x:v>
+        <x:v>结束时间</x:v>
       </x:c>
       <x:c r="T1" s="14" t="str">
-        <x:v>结束时间</x:v>
+        <x:v>通话状态</x:v>
       </x:c>
       <x:c r="U1" s="14" t="str">
-        <x:v>通话状态</x:v>
+        <x:v>通话结果</x:v>
       </x:c>
       <x:c r="V1" s="14" t="str">
-        <x:v>通话结果</x:v>
+        <x:v>接通时长（秒）</x:v>
       </x:c>
       <x:c r="W1" s="14" t="str">
-        <x:v>接通时长（秒）</x:v>
+        <x:v>结束原因</x:v>
       </x:c>
       <x:c r="X1" s="14" t="str">
-        <x:v>结束原因</x:v>
+        <x:v>同步时间</x:v>
       </x:c>
       <x:c r="Y1" s="14" t="str">
-        <x:v>同步时间</x:v>
-      </x:c>
-      <x:c r="Z1" s="14" t="str">
         <x:v>通话备注</x:v>
       </x:c>
     </x:row>
@@ -1253,11 +1225,11 @@
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
-      <x:c r="I2" s="4"/>
-      <x:c r="J2" s="15"/>
-      <x:c r="K2" s="4"/>
+      <x:c r="I2" s="15"/>
+      <x:c r="J2" s="4"/>
+      <x:c r="K2" s="15"/>
       <x:c r="L2" s="15"/>
-      <x:c r="M2" s="15"/>
+      <x:c r="M2" s="4"/>
       <x:c r="N2" s="4"/>
       <x:c r="O2" s="4"/>
       <x:c r="P2" s="4"/>
@@ -1270,7 +1242,6 @@
       <x:c r="W2" s="4"/>
       <x:c r="X2" s="4"/>
       <x:c r="Y2" s="4"/>
-      <x:c r="Z2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -1281,11 +1252,11 @@
       <x:c r="F3" s="4"/>
       <x:c r="G3" s="4"/>
       <x:c r="H3" s="4"/>
-      <x:c r="I3" s="4"/>
-      <x:c r="J3" s="15"/>
-      <x:c r="K3" s="4"/>
+      <x:c r="I3" s="15"/>
+      <x:c r="J3" s="4"/>
+      <x:c r="K3" s="15"/>
       <x:c r="L3" s="15"/>
-      <x:c r="M3" s="15"/>
+      <x:c r="M3" s="4"/>
       <x:c r="N3" s="4"/>
       <x:c r="O3" s="4"/>
       <x:c r="P3" s="4"/>
@@ -1298,7 +1269,6 @@
       <x:c r="W3" s="4"/>
       <x:c r="X3" s="4"/>
       <x:c r="Y3" s="4"/>
-      <x:c r="Z3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1327,7 +1297,6 @@
     <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1344,48 +1313,45 @@
         <x:v>用户类型</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
+        <x:v>当前 CC 账号</x:v>
       </x:c>
       <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
+        <x:v>注册时间</x:v>
       </x:c>
       <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
+        <x:v>注册日期</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
+        <x:v>用户状态</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
+        <x:v>订单 ID</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>订单 ID</x:v>
+        <x:v>商品名称</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>商品名称</x:v>
+        <x:v>订单状态</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>订单状态</x:v>
+        <x:v>原价</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>原价</x:v>
+        <x:v>实付金额</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>实付金额</x:v>
+        <x:v>币种</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>币种</x:v>
+        <x:v>支付方式</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>支付方式</x:v>
+        <x:v>支付时间</x:v>
       </x:c>
       <x:c r="Q1" s="14" t="str">
-        <x:v>支付时间</x:v>
+        <x:v>支付日期</x:v>
       </x:c>
       <x:c r="R1" s="14" t="str">
-        <x:v>支付日期</x:v>
-      </x:c>
-      <x:c r="S1" s="14" t="str">
         <x:v>有效期截止时间</x:v>
       </x:c>
     </x:row>
@@ -1398,8 +1364,8 @@
       <x:c r="F2" s="4"/>
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
-      <x:c r="I2" s="4"/>
-      <x:c r="J2" s="15"/>
+      <x:c r="I2" s="15"/>
+      <x:c r="J2" s="4"/>
       <x:c r="K2" s="4"/>
       <x:c r="L2" s="4"/>
       <x:c r="M2" s="4"/>
@@ -1408,7 +1374,6 @@
       <x:c r="P2" s="4"/>
       <x:c r="Q2" s="4"/>
       <x:c r="R2" s="4"/>
-      <x:c r="S2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -1419,8 +1384,8 @@
       <x:c r="F3" s="4"/>
       <x:c r="G3" s="4"/>
       <x:c r="H3" s="4"/>
-      <x:c r="I3" s="4"/>
-      <x:c r="J3" s="15"/>
+      <x:c r="I3" s="15"/>
+      <x:c r="J3" s="4"/>
       <x:c r="K3" s="4"/>
       <x:c r="L3" s="4"/>
       <x:c r="M3" s="4"/>
@@ -1429,7 +1394,6 @@
       <x:c r="P3" s="4"/>
       <x:c r="Q3" s="4"/>
       <x:c r="R3" s="4"/>
-      <x:c r="S3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1456,7 +1420,6 @@
     <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="48" customHeight="1">
@@ -1473,42 +1436,39 @@
         <x:v>用户类型</x:v>
       </x:c>
       <x:c r="E1" s="14" t="str">
-        <x:v>当前 CC</x:v>
+        <x:v>当前 CC 账号</x:v>
       </x:c>
       <x:c r="F1" s="14" t="str">
-        <x:v>当前 CC 账号</x:v>
+        <x:v>注册时间</x:v>
       </x:c>
       <x:c r="G1" s="14" t="str">
-        <x:v>注册时间</x:v>
+        <x:v>注册日期</x:v>
       </x:c>
       <x:c r="H1" s="14" t="str">
-        <x:v>注册日期</x:v>
+        <x:v>用户状态</x:v>
       </x:c>
       <x:c r="I1" s="14" t="str">
-        <x:v>用户状态</x:v>
+        <x:v>当前销售阶段</x:v>
       </x:c>
       <x:c r="J1" s="14" t="str">
-        <x:v>当前销售阶段</x:v>
+        <x:v>原因分类</x:v>
       </x:c>
       <x:c r="K1" s="14" t="str">
-        <x:v>原因分类</x:v>
+        <x:v>具体原因</x:v>
       </x:c>
       <x:c r="L1" s="14" t="str">
-        <x:v>具体原因</x:v>
+        <x:v>拒绝或结束时间</x:v>
       </x:c>
       <x:c r="M1" s="14" t="str">
-        <x:v>拒绝或结束时间</x:v>
+        <x:v>拒绝或结束日期</x:v>
       </x:c>
       <x:c r="N1" s="14" t="str">
-        <x:v>拒绝或结束日期</x:v>
+        <x:v>时间依据</x:v>
       </x:c>
       <x:c r="O1" s="14" t="str">
-        <x:v>时间依据</x:v>
+        <x:v>最近跟进时间</x:v>
       </x:c>
       <x:c r="P1" s="14" t="str">
-        <x:v>最近跟进时间</x:v>
-      </x:c>
-      <x:c r="Q1" s="14" t="str">
         <x:v>最近跟进备注</x:v>
       </x:c>
     </x:row>
@@ -1529,7 +1489,6 @@
       <x:c r="N2" s="4"/>
       <x:c r="O2" s="4"/>
       <x:c r="P2" s="4"/>
-      <x:c r="Q2" s="4"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="15"/>
@@ -1548,7 +1507,6 @@
       <x:c r="N3" s="4"/>
       <x:c r="O3" s="4"/>
       <x:c r="P3" s="4"/>
-      <x:c r="Q3" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>